<commit_message>
feat: async ingestion, search_time, inference_time, db_ingestion
</commit_message>
<xml_diff>
--- a/marcelo_benchmark_results.xlsx
+++ b/marcelo_benchmark_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marce\Desktop\Code\NLP_Assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72D6221-73BE-493D-94C5-3C6B14F2B103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649EC6B6-9955-4C76-B8E3-22FFDB571FC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="69">
   <si>
     <t>experiment_id</t>
   </si>
@@ -82,6 +82,36 @@
     <t>timestamp</t>
   </si>
   <si>
+    <t>mean_search_time</t>
+  </si>
+  <si>
+    <t>mean_reasoning_time</t>
+  </si>
+  <si>
+    <t>entertainment_mean_search_time</t>
+  </si>
+  <si>
+    <t>entertainment_mean_reasoning_time</t>
+  </si>
+  <si>
+    <t>science_nature_mean_search_time</t>
+  </si>
+  <si>
+    <t>science_nature_mean_reasoning_time</t>
+  </si>
+  <si>
+    <t>ancient_history_mean_search_time</t>
+  </si>
+  <si>
+    <t>ancient_history_mean_reasoning_time</t>
+  </si>
+  <si>
+    <t>maths_mean_search_time</t>
+  </si>
+  <si>
+    <t>maths_mean_reasoning_time</t>
+  </si>
+  <si>
     <t>6f222b8968774e979b341f21acf72be3</t>
   </si>
   <si>
@@ -101,6 +131,102 @@
   </si>
   <si>
     <t>2026-05-06 15:06:27</t>
+  </si>
+  <si>
+    <t>23b7589c755749d6b7b0d32ff96e206d</t>
+  </si>
+  <si>
+    <t>2026-05-07 12:16:27</t>
+  </si>
+  <si>
+    <t>303af31b0a3446288710d1e9cc37e62e</t>
+  </si>
+  <si>
+    <t>Try with small database only for history.</t>
+  </si>
+  <si>
+    <t>2026-05-10 13:28:16</t>
+  </si>
+  <si>
+    <t>992f34dd6b8b44f2bb05aaaf364c813b</t>
+  </si>
+  <si>
+    <t>2026-05-10 13:44:32</t>
+  </si>
+  <si>
+    <t>3e4f75ea03004483816427243e5b9668</t>
+  </si>
+  <si>
+    <t>2026-05-10 13:55:03</t>
+  </si>
+  <si>
+    <t>5178452549834fed8b9c71f02e31b2dc</t>
+  </si>
+  <si>
+    <t>2026-05-10 13:57:52</t>
+  </si>
+  <si>
+    <t>5f994b310d2746da845f61533e779981</t>
+  </si>
+  <si>
+    <t>2026-05-10 14:00:06</t>
+  </si>
+  <si>
+    <t>bfcbf0acdb244012be2819ca5e933b79</t>
+  </si>
+  <si>
+    <t>2026-05-10 16:45:06</t>
+  </si>
+  <si>
+    <t>cfc6d3a205dd43139e5e7759ae811cbc</t>
+  </si>
+  <si>
+    <t>2026-05-10 17:38:12</t>
+  </si>
+  <si>
+    <t>25aff2756d8b45cd9f92252bf11320b5</t>
+  </si>
+  <si>
+    <t>Try with small database for all cases.</t>
+  </si>
+  <si>
+    <t>2026-05-10 18:12:18</t>
+  </si>
+  <si>
+    <t>b46b23112b244e7086e955e3a49bba9b</t>
+  </si>
+  <si>
+    <t>Try with 1000 articles on database for all cases.</t>
+  </si>
+  <si>
+    <t>2026-05-11 06:15:28</t>
+  </si>
+  <si>
+    <t>31bba39f11b042eb9b1dcaf1987f2f04</t>
+  </si>
+  <si>
+    <t>Try with 1000 articles on database for all cases. Science has 12000</t>
+  </si>
+  <si>
+    <t>2026-05-11 07:31:29</t>
+  </si>
+  <si>
+    <t>bfa54c7919c7429bb7411d5c37214b40</t>
+  </si>
+  <si>
+    <t>RAG. Science, Entertainment have 17k articles, math 10k, History 5k</t>
+  </si>
+  <si>
+    <t>2026-05-11 11:37:52</t>
+  </si>
+  <si>
+    <t>64b171f5cf7d431abc42704789a7dab1</t>
+  </si>
+  <si>
+    <t>gemma2</t>
+  </si>
+  <si>
+    <t>2026-05-11 12:04:09</t>
   </si>
 </sst>
 </file>
@@ -463,20 +589,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:AD15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="31.46484375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.46484375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.19921875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.53125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.73046875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="23" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="34.53125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.3984375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="34.9296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="35.265625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.06640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="27.59765625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.06640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="32.46484375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -537,22 +667,52 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -561,7 +721,7 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="I2">
         <v>0.2</v>
@@ -597,7 +757,1113 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>26</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3">
+        <v>0.2</v>
+      </c>
+      <c r="J3">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="K3">
+        <v>10.23879445923699</v>
+      </c>
+      <c r="L3">
+        <v>13.22459173202515</v>
+      </c>
+      <c r="M3">
+        <v>0.8</v>
+      </c>
+      <c r="N3">
+        <v>13.013095736503599</v>
+      </c>
+      <c r="O3">
+        <v>0.5</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4">
+        <v>0.2</v>
+      </c>
+      <c r="J4">
+        <v>0.42857142857142849</v>
+      </c>
+      <c r="K4">
+        <v>4.5340960366385321</v>
+      </c>
+      <c r="L4">
+        <v>5.6097428003946943</v>
+      </c>
+      <c r="M4">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>7.4547219276428223</v>
+      </c>
+      <c r="S4">
+        <v>0.5</v>
+      </c>
+      <c r="T4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5">
+        <v>0.2</v>
+      </c>
+      <c r="J5">
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="K5">
+        <v>6.5261556885459209</v>
+      </c>
+      <c r="L5">
+        <v>7.202437162399292</v>
+      </c>
+      <c r="M5">
+        <v>0.5</v>
+      </c>
+      <c r="N5">
+        <v>2.5760774612426758</v>
+      </c>
+      <c r="O5">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="P5">
+        <v>32.783676624298103</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>6.5666193962097168</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6">
+        <v>0.2</v>
+      </c>
+      <c r="J6">
+        <v>0.42857142857142849</v>
+      </c>
+      <c r="K6">
+        <v>8.8454953261784137</v>
+      </c>
+      <c r="L6">
+        <v>10.607508659362789</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>3.372485876083374</v>
+      </c>
+      <c r="O6">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="P6">
+        <v>33.301580905914307</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>3.9459600448608398</v>
+      </c>
+      <c r="S6">
+        <v>0.5</v>
+      </c>
+      <c r="T6" t="s">
+        <v>45</v>
+      </c>
+      <c r="U6">
+        <v>1.430264064243862</v>
+      </c>
+      <c r="V6">
+        <v>3.61935349873134</v>
+      </c>
+      <c r="W6">
+        <v>2.6166706085205078</v>
+      </c>
+      <c r="X6">
+        <v>7.1404488086700439</v>
+      </c>
+      <c r="Y6">
+        <v>0.81333231925964355</v>
+      </c>
+      <c r="Z6">
+        <v>2.1305034160614009</v>
+      </c>
+      <c r="AA6">
+        <v>2.6166706085205078</v>
+      </c>
+      <c r="AB6">
+        <v>7.1404488086700439</v>
+      </c>
+      <c r="AC6">
+        <v>1.169255137443542</v>
+      </c>
+      <c r="AD6">
+        <v>2.3315333127975459</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7">
+        <v>0.2</v>
+      </c>
+      <c r="J7">
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="K7">
+        <v>6.5736239173195576</v>
+      </c>
+      <c r="L7">
+        <v>2.3451036385127479</v>
+      </c>
+      <c r="M7">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="N7">
+        <v>8.3019819259643555</v>
+      </c>
+      <c r="O7">
+        <v>0.5</v>
+      </c>
+      <c r="P7">
+        <v>33.099678039550781</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>6.1904957294464111</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7" t="s">
+        <v>47</v>
+      </c>
+      <c r="U7">
+        <v>1.312012737447565</v>
+      </c>
+      <c r="V7">
+        <v>4.8253350257873544</v>
+      </c>
+      <c r="W7">
+        <v>0.41938229969569613</v>
+      </c>
+      <c r="X7">
+        <v>1.802048138209752</v>
+      </c>
+      <c r="Y7">
+        <v>3.546663761138916</v>
+      </c>
+      <c r="Z7">
+        <v>3.900126695632935</v>
+      </c>
+      <c r="AA7">
+        <v>2.241461038589478</v>
+      </c>
+      <c r="AB7">
+        <v>30.00133037567139</v>
+      </c>
+      <c r="AC7">
+        <v>2.1616754531860352</v>
+      </c>
+      <c r="AD7">
+        <v>2.6627645492553711</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8">
+        <v>0.2</v>
+      </c>
+      <c r="J8">
+        <v>0.6</v>
+      </c>
+      <c r="K8">
+        <v>10.277619481086729</v>
+      </c>
+      <c r="L8">
+        <v>9.2049137592315677</v>
+      </c>
+      <c r="M8">
+        <v>0.8</v>
+      </c>
+      <c r="N8">
+        <v>5.6406026681264239</v>
+      </c>
+      <c r="O8">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="P8">
+        <v>33.456361055374153</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>6.3734569549560547</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8" t="s">
+        <v>49</v>
+      </c>
+      <c r="U8">
+        <v>4.4869028091430661</v>
+      </c>
+      <c r="V8">
+        <v>5.3190570831298816</v>
+      </c>
+      <c r="W8">
+        <v>6.4823586463928224</v>
+      </c>
+      <c r="X8">
+        <v>2.5405254840850828</v>
+      </c>
+      <c r="Y8">
+        <v>2.658977429072062</v>
+      </c>
+      <c r="Z8">
+        <v>2.5262384414672852</v>
+      </c>
+      <c r="AA8">
+        <v>2.2728126049041748</v>
+      </c>
+      <c r="AB8">
+        <v>30.00607872009277</v>
+      </c>
+      <c r="AC8">
+        <v>2.207489967346191</v>
+      </c>
+      <c r="AD8">
+        <v>2.9031493663787842</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9">
+        <v>0.2</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>40.316687603791557</v>
+      </c>
+      <c r="L9">
+        <v>29.429561932881668</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>45.43484822909037</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>40.445159832636513</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>45.957180420557663</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9" t="s">
+        <v>51</v>
+      </c>
+      <c r="U9">
+        <v>9.1038258671760559</v>
+      </c>
+      <c r="V9">
+        <v>29.526614884535469</v>
+      </c>
+      <c r="W9">
+        <v>7.2017890612284354</v>
+      </c>
+      <c r="X9">
+        <v>21.936750411987301</v>
+      </c>
+      <c r="Y9">
+        <v>12.946824630101521</v>
+      </c>
+      <c r="Z9">
+        <v>32.053855498631798</v>
+      </c>
+      <c r="AA9">
+        <v>7.714528401692708</v>
+      </c>
+      <c r="AB9">
+        <v>32.046004215876259</v>
+      </c>
+      <c r="AC9">
+        <v>8.5521613756815587</v>
+      </c>
+      <c r="AD9">
+        <v>32.069849411646523</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>35</v>
+      </c>
+      <c r="I10">
+        <v>0.2</v>
+      </c>
+      <c r="J10">
+        <v>0.14285714285714279</v>
+      </c>
+      <c r="K10">
+        <v>35.059031622750418</v>
+      </c>
+      <c r="L10">
+        <v>25.870357084274289</v>
+      </c>
+      <c r="M10">
+        <v>0.4</v>
+      </c>
+      <c r="N10">
+        <v>43.923736413319908</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>35.964944918950401</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>40.602871100107834</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10" t="s">
+        <v>53</v>
+      </c>
+      <c r="U10">
+        <v>6.1621383769171576</v>
+      </c>
+      <c r="V10">
+        <v>28.301041926656449</v>
+      </c>
+      <c r="W10">
+        <v>3.9147161483764652</v>
+      </c>
+      <c r="X10">
+        <v>21.56548347473144</v>
+      </c>
+      <c r="Y10">
+        <v>10.566285610198969</v>
+      </c>
+      <c r="Z10">
+        <v>32.040262699127197</v>
+      </c>
+      <c r="AA10">
+        <v>3.536852121353149</v>
+      </c>
+      <c r="AB10">
+        <v>32.048989057540886</v>
+      </c>
+      <c r="AC10">
+        <v>8.1289811134338379</v>
+      </c>
+      <c r="AD10">
+        <v>32.039804776509612</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11">
+        <v>0.2</v>
+      </c>
+      <c r="J11">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="K11">
+        <v>21.28913357522752</v>
+      </c>
+      <c r="L11">
+        <v>11.2480001449585</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>26.80850267410278</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>24.796290636062619</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>21.96553842226664</v>
+      </c>
+      <c r="S11">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="T11" t="s">
+        <v>56</v>
+      </c>
+      <c r="U11">
+        <v>5.5621363586849633</v>
+      </c>
+      <c r="V11">
+        <v>14.823449320263331</v>
+      </c>
+      <c r="W11">
+        <v>2.4002759456634521</v>
+      </c>
+      <c r="X11">
+        <v>7.8465733528137207</v>
+      </c>
+      <c r="Y11">
+        <v>9.2791532278060913</v>
+      </c>
+      <c r="Z11">
+        <v>16.525686740875241</v>
+      </c>
+      <c r="AA11">
+        <v>8.0294733047485352</v>
+      </c>
+      <c r="AB11">
+        <v>15.71383714675903</v>
+      </c>
+      <c r="AC11">
+        <v>3.5471407572428379</v>
+      </c>
+      <c r="AD11">
+        <v>17.746283133824669</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12">
+        <v>0.2</v>
+      </c>
+      <c r="J12">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="K12">
+        <v>17.660133401552841</v>
+      </c>
+      <c r="L12">
+        <v>11.4475508928299</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>14.43164806365967</v>
+      </c>
+      <c r="O12">
+        <v>0.6</v>
+      </c>
+      <c r="P12">
+        <v>28.977506081263229</v>
+      </c>
+      <c r="Q12">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="R12">
+        <v>14.967870235443121</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12" t="s">
+        <v>59</v>
+      </c>
+      <c r="U12">
+        <v>4.8513692617416382</v>
+      </c>
+      <c r="V12">
+        <v>12.50164008140564</v>
+      </c>
+      <c r="W12">
+        <v>2.8473677635192871</v>
+      </c>
+      <c r="X12">
+        <v>8.1352723836898804</v>
+      </c>
+      <c r="Y12">
+        <v>3.3641745567321779</v>
+      </c>
+      <c r="Z12">
+        <v>10.8455659866333</v>
+      </c>
+      <c r="AA12">
+        <v>10.27377430597941</v>
+      </c>
+      <c r="AB12">
+        <v>18.416534264882401</v>
+      </c>
+      <c r="AC12">
+        <v>2.439749956130981</v>
+      </c>
+      <c r="AD12">
+        <v>12.135851740837101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13">
+        <v>0.2</v>
+      </c>
+      <c r="J13">
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="K13">
+        <v>14.4281784621152</v>
+      </c>
+      <c r="L13">
+        <v>13.40805661678314</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>6.0666224360466003</v>
+      </c>
+      <c r="O13">
+        <v>0.5</v>
+      </c>
+      <c r="P13">
+        <v>13.076462507247919</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>27.158145030339561</v>
+      </c>
+      <c r="S13">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="T13" t="s">
+        <v>62</v>
+      </c>
+      <c r="U13">
+        <v>4.2973682230169121</v>
+      </c>
+      <c r="V13">
+        <v>9.7663225910880342</v>
+      </c>
+      <c r="W13">
+        <v>2.437616109848022</v>
+      </c>
+      <c r="X13">
+        <v>10.54658615589142</v>
+      </c>
+      <c r="Y13">
+        <v>1.2806392908096309</v>
+      </c>
+      <c r="Z13">
+        <v>4.4764740467071533</v>
+      </c>
+      <c r="AA13">
+        <v>1.300129771232605</v>
+      </c>
+      <c r="AB13">
+        <v>11.351382255554199</v>
+      </c>
+      <c r="AC13">
+        <v>11.557667175928749</v>
+      </c>
+      <c r="AD13">
+        <v>15.24257183074951</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="s">
+        <v>35</v>
+      </c>
+      <c r="I14">
+        <v>0.2</v>
+      </c>
+      <c r="J14">
+        <v>0.31034482758620691</v>
+      </c>
+      <c r="K14">
+        <v>9.4199826470736792</v>
+      </c>
+      <c r="L14">
+        <v>9.1039079030354824</v>
+      </c>
+      <c r="M14">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="N14">
+        <v>5.7921375698513451</v>
+      </c>
+      <c r="O14">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="P14">
+        <v>3.3865915536880489</v>
+      </c>
+      <c r="Q14">
+        <v>0.16666666666666671</v>
+      </c>
+      <c r="R14">
+        <v>23.7591076374054</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14" t="s">
+        <v>65</v>
+      </c>
+      <c r="U14">
+        <v>3.0604558402094351</v>
+      </c>
+      <c r="V14">
+        <v>6.213400331036798</v>
+      </c>
+      <c r="W14">
+        <v>2.924188031090631</v>
+      </c>
+      <c r="X14">
+        <v>6.0843899779849586</v>
+      </c>
+      <c r="Y14">
+        <v>1.4152988857693141</v>
+      </c>
+      <c r="Z14">
+        <v>4.2450689739651146</v>
+      </c>
+      <c r="AA14">
+        <v>0.60805976390838623</v>
+      </c>
+      <c r="AB14">
+        <v>2.584495703379313</v>
+      </c>
+      <c r="AC14">
+        <v>9.2098957061767575</v>
+      </c>
+      <c r="AD14">
+        <v>14.34330096244812</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15">
+        <v>9</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="s">
+        <v>35</v>
+      </c>
+      <c r="I15">
+        <v>0.2</v>
+      </c>
+      <c r="J15">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="K15">
+        <v>21.078132838913891</v>
+      </c>
+      <c r="L15">
+        <v>15.286365733427161</v>
+      </c>
+      <c r="M15">
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="N15">
+        <v>30.438118600845339</v>
+      </c>
+      <c r="O15">
+        <v>0.5</v>
+      </c>
+      <c r="P15">
+        <v>18.641124248504639</v>
+      </c>
+      <c r="Q15">
+        <v>0.6875</v>
+      </c>
+      <c r="R15">
+        <v>44.796859741210938</v>
+      </c>
+      <c r="S15">
+        <v>0.16666666666666671</v>
+      </c>
+      <c r="T15" t="s">
+        <v>68</v>
+      </c>
+      <c r="U15">
+        <v>5.5603789669094663</v>
+      </c>
+      <c r="V15">
+        <v>15.40473222010063</v>
+      </c>
+      <c r="W15">
+        <v>5.4125340756248024</v>
+      </c>
+      <c r="X15">
+        <v>9.8080087128807509</v>
+      </c>
+      <c r="Y15">
+        <v>6.3740124464035031</v>
+      </c>
+      <c r="Z15">
+        <v>23.940307807922359</v>
+      </c>
+      <c r="AA15">
+        <v>5.6049143224954614</v>
+      </c>
+      <c r="AB15">
+        <v>12.922544315457341</v>
+      </c>
+      <c r="AC15">
+        <v>4.9233499368031817</v>
+      </c>
+      <c r="AD15">
+        <v>39.512707193692528</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: science,history,entertainment improvement (math 0% still because of timeout).
</commit_message>
<xml_diff>
--- a/marcelo_benchmark_results.xlsx
+++ b/marcelo_benchmark_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marce\Desktop\Code\NLP_Assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649EC6B6-9955-4C76-B8E3-22FFDB571FC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE825686-34B4-4222-9768-80246B79A709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="77">
   <si>
     <t>experiment_id</t>
   </si>
@@ -227,6 +227,30 @@
   </si>
   <si>
     <t>2026-05-11 12:04:09</t>
+  </si>
+  <si>
+    <t>4c5c326bfff64ba48e960ca984776b3b</t>
+  </si>
+  <si>
+    <t>RAG. Science, Entertainment have 17k articles, math better prompt, History 5k</t>
+  </si>
+  <si>
+    <t>2026-05-11 15:33:42</t>
+  </si>
+  <si>
+    <t>c424fcbad2294f058f188cd95f3f5888</t>
+  </si>
+  <si>
+    <t>RAG. Science, Entertainment have 17k articles, math with CoT prompt, History 5k</t>
+  </si>
+  <si>
+    <t>2026-05-11 15:53:36</t>
+  </si>
+  <si>
+    <t>bd386a0b63714fa0a6ba05660c68c2ce</t>
+  </si>
+  <si>
+    <t>2026-05-11 17:42:46</t>
   </si>
 </sst>
 </file>
@@ -589,21 +613,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD15"/>
+  <dimension ref="A1:AD18"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="10" max="10" width="21.53125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="34.53125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="34.9296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="35.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.3984375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.06640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="27.59765625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.265625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.06640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="32.46484375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="22.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.45">
@@ -1864,6 +1882,282 @@
       </c>
       <c r="AD15">
         <v>39.512707193692528</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16">
+        <v>5</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16">
+        <v>0.2</v>
+      </c>
+      <c r="J16">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="K16">
+        <v>22.43148280183474</v>
+      </c>
+      <c r="L16">
+        <v>17.350332319736481</v>
+      </c>
+      <c r="M16">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N16">
+        <v>32.371471563975007</v>
+      </c>
+      <c r="O16">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="P16">
+        <v>14.785202741622919</v>
+      </c>
+      <c r="Q16">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="R16">
+        <v>64.770382761955261</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16" t="s">
+        <v>71</v>
+      </c>
+      <c r="U16">
+        <v>5.3406893511613207</v>
+      </c>
+      <c r="V16">
+        <v>16.753254512945809</v>
+      </c>
+      <c r="W16">
+        <v>5.6401225328445426</v>
+      </c>
+      <c r="X16">
+        <v>11.64361310005188</v>
+      </c>
+      <c r="Y16">
+        <v>6.9332546393076582</v>
+      </c>
+      <c r="Z16">
+        <v>24.680554628372189</v>
+      </c>
+      <c r="AA16">
+        <v>4.9518047400883267</v>
+      </c>
+      <c r="AB16">
+        <v>9.4927732603890558</v>
+      </c>
+      <c r="AC16">
+        <v>2.516338467597961</v>
+      </c>
+      <c r="AD16">
+        <v>60.931837201118469</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17">
+        <v>5</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="s">
+        <v>35</v>
+      </c>
+      <c r="I17">
+        <v>0.2</v>
+      </c>
+      <c r="J17">
+        <v>0.72413793103448276</v>
+      </c>
+      <c r="K17">
+        <v>21.832084137817908</v>
+      </c>
+      <c r="L17">
+        <v>18.994759440422062</v>
+      </c>
+      <c r="M17">
+        <v>0.5</v>
+      </c>
+      <c r="N17">
+        <v>27.021135282516479</v>
+      </c>
+      <c r="O17">
+        <v>0.6</v>
+      </c>
+      <c r="P17">
+        <v>17.620497756534149</v>
+      </c>
+      <c r="Q17">
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="R17">
+        <v>52.438383102416992</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17" t="s">
+        <v>74</v>
+      </c>
+      <c r="U17">
+        <v>6.4390871442597488</v>
+      </c>
+      <c r="V17">
+        <v>15.186037088262619</v>
+      </c>
+      <c r="W17">
+        <v>2.3462901711463928</v>
+      </c>
+      <c r="X17">
+        <v>16.433293700218201</v>
+      </c>
+      <c r="Y17">
+        <v>3.3699151992797849</v>
+      </c>
+      <c r="Z17">
+        <v>23.14219498634338</v>
+      </c>
+      <c r="AA17">
+        <v>8.657617449760437</v>
+      </c>
+      <c r="AB17">
+        <v>8.8836905029084949</v>
+      </c>
+      <c r="AC17">
+        <v>2.3308382034301758</v>
+      </c>
+      <c r="AD17">
+        <v>49.522248387336731</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18">
+        <v>5</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="s">
+        <v>35</v>
+      </c>
+      <c r="I18">
+        <v>0.2</v>
+      </c>
+      <c r="J18">
+        <v>0.76470588235294112</v>
+      </c>
+      <c r="K18">
+        <v>17.624478728163481</v>
+      </c>
+      <c r="L18">
+        <v>16.729106575250629</v>
+      </c>
+      <c r="M18">
+        <v>0.625</v>
+      </c>
+      <c r="N18">
+        <v>17.44653582572937</v>
+      </c>
+      <c r="O18">
+        <v>0.85</v>
+      </c>
+      <c r="P18">
+        <v>13.2111967086792</v>
+      </c>
+      <c r="Q18">
+        <v>0.85</v>
+      </c>
+      <c r="R18">
+        <v>50.620303948720299</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18" t="s">
+        <v>76</v>
+      </c>
+      <c r="U18">
+        <v>3.9063346339207068</v>
+      </c>
+      <c r="V18">
+        <v>13.635130597095859</v>
+      </c>
+      <c r="W18">
+        <v>5.2995361983776093</v>
+      </c>
+      <c r="X18">
+        <v>11.32486632466316</v>
+      </c>
+      <c r="Y18">
+        <v>4.1285791039466861</v>
+      </c>
+      <c r="Z18">
+        <v>13.26141041517258</v>
+      </c>
+      <c r="AA18">
+        <v>2.3079854249954219</v>
+      </c>
+      <c r="AB18">
+        <v>10.845223438739779</v>
+      </c>
+      <c r="AC18">
+        <v>9.3651620546976719</v>
+      </c>
+      <c r="AD18">
+        <v>40.886684258778892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>